<commit_message>
Rate model: descriptive bs_side column; asset rows may leave beta/margin blank, liability rows must set beta
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/balance_gen_add_data/input/interest_rt.xlsx
+++ b/balance_gen_add_data/input/interest_rt.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -433,30 +433,35 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>bs_side</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>beta</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>margin_pct</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>index_floor</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>client_floor</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>index_cap</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>client_cap</t>
         </is>
@@ -469,18 +474,23 @@
       <c r="B2" t="n">
         <v>6000</v>
       </c>
-      <c r="C2" t="n">
-        <v>0</v>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
       <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -489,18 +499,23 @@
       <c r="B3" t="n">
         <v>7060</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
         <v>0.75</v>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
         <v>0.5</v>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
       <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
@@ -509,18 +524,23 @@
       <c r="B4" t="n">
         <v>8000</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
         <v>0.6</v>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>0.12</v>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
       <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
@@ -529,18 +549,23 @@
       <c r="B5" t="n">
         <v>1000</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
         <v>1</v>
       </c>
-      <c r="D5" t="n">
-        <v>0</v>
-      </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
-      <c r="F5" t="inlineStr"/>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
@@ -549,18 +574,23 @@
       <c r="B6" t="n">
         <v>1100</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
         <v>1</v>
       </c>
-      <c r="D6" t="n">
-        <v>0</v>
-      </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
-      <c r="F6" t="inlineStr"/>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
@@ -569,18 +599,23 @@
       <c r="B7" t="n">
         <v>2000</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
         <v>1</v>
       </c>
-      <c r="D7" t="n">
-        <v>0</v>
-      </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
-      <c r="F7" t="inlineStr"/>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
@@ -589,18 +624,23 @@
       <c r="B8" t="n">
         <v>2100</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
         <v>1</v>
       </c>
-      <c r="D8" t="n">
-        <v>0</v>
-      </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
-      <c r="F8" t="inlineStr"/>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
@@ -609,18 +649,23 @@
       <c r="B9" t="n">
         <v>3000</v>
       </c>
-      <c r="C9" t="n">
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
         <v>1</v>
       </c>
-      <c r="D9" t="n">
-        <v>0</v>
-      </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
-      <c r="F9" t="inlineStr"/>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
@@ -629,18 +674,23 @@
       <c r="B10" t="n">
         <v>3100</v>
       </c>
-      <c r="C10" t="n">
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
         <v>1</v>
       </c>
-      <c r="D10" t="n">
-        <v>0</v>
-      </c>
       <c r="E10" t="n">
         <v>0</v>
       </c>
-      <c r="F10" t="inlineStr"/>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
@@ -649,18 +699,23 @@
       <c r="B11" t="n">
         <v>4100</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
         <v>0.8</v>
       </c>
-      <c r="D11" t="n">
-        <v>0</v>
-      </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
-      <c r="F11" t="inlineStr"/>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
@@ -669,18 +724,23 @@
       <c r="B12" t="n">
         <v>5000</v>
       </c>
-      <c r="C12" t="n">
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
         <v>1</v>
       </c>
-      <c r="D12" t="n">
-        <v>0</v>
-      </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
-      <c r="F12" t="inlineStr"/>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
@@ -689,18 +749,23 @@
       <c r="B13" t="n">
         <v>7900</v>
       </c>
-      <c r="C13" t="n">
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>A/L</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
         <v>1</v>
       </c>
-      <c r="D13" t="n">
-        <v>0</v>
-      </c>
       <c r="E13" t="n">
         <v>0</v>
       </c>
-      <c r="F13" t="inlineStr"/>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
@@ -709,18 +774,23 @@
       <c r="B14" t="n">
         <v>6300</v>
       </c>
-      <c r="C14" t="n">
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
         <v>0.1</v>
       </c>
-      <c r="D14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="n">
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="n">
         <v>0.001</v>
       </c>
     </row>
@@ -731,18 +801,23 @@
       <c r="B15" t="n">
         <v>3200</v>
       </c>
-      <c r="C15" t="n">
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
         <v>1</v>
       </c>
-      <c r="D15" t="n">
+      <c r="E15" t="n">
         <v>-0.75</v>
       </c>
-      <c r="E15" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" t="inlineStr"/>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>